<commit_message>
Data Visualisations and demo notebook
</commit_message>
<xml_diff>
--- a/Results/CIFAR-10/CIFAR-10_Full_Results.xlsx
+++ b/Results/CIFAR-10/CIFAR-10_Full_Results.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lewis/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniofnottm-my.sharepoint.com/personal/psyle2_nottingham_ac_uk/Documents/Year 3/Dissertation/Programming/Repo/Diss-Notebook/Results/CIFAR-10/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5D4160E4-F07F-334F-A5A6-BB3262A1B01C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="8_{5D4160E4-F07F-334F-A5A6-BB3262A1B01C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5A8B6C8B-B1BE-C247-BF4C-C9B0B66C7080}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4420" yWindow="660" windowWidth="25820" windowHeight="17700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="683" uniqueCount="110">
   <si>
     <t>model</t>
   </si>
@@ -347,6 +347,9 @@
   </si>
   <si>
     <t>resnet50_cifar10</t>
+  </si>
+  <si>
+    <t>Column1</t>
   </si>
 </sst>
 </file>
@@ -365,6 +368,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -411,7 +415,72 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -422,6 +491,48 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E9404C44-DB89-DA4A-A469-B4F5294E1613}" name="Table1" displayName="Table1" ref="A1:M177" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:M177" xr:uid="{E9404C44-DB89-DA4A-A469-B4F5294E1613}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="apgd -&gt; jpeg    (eps=0.03, 25%)"/>
+        <filter val="apgd -&gt; jpeg    (eps=0.03, 50%)"/>
+        <filter val="apgd -&gt; jpeg    (eps=0.03, 75%)"/>
+        <filter val="apgd -&gt; jpeg2000    (eps=0.03, 25%)"/>
+        <filter val="apgd -&gt; jpeg2000    (eps=0.03, 50%)"/>
+        <filter val="apgd -&gt; jpeg2000    (eps=0.03, 75%)"/>
+        <filter val="apgd -&gt; patchsvd    (eps=0.03, 25%)"/>
+        <filter val="apgd -&gt; patchsvd    (eps=0.03, 50%)"/>
+        <filter val="apgd -&gt; patchsvd    (eps=0.03, 75%)"/>
+        <filter val="apgd -&gt; pca    (eps=0.03, 25%)"/>
+        <filter val="apgd -&gt; pca    (eps=0.03, 50%)"/>
+        <filter val="apgd -&gt; pca    (eps=0.03, 75%)"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A78:M177">
+    <sortCondition ref="H1:H177"/>
+  </sortState>
+  <tableColumns count="13">
+    <tableColumn id="1" xr3:uid="{5B4762F2-BFC0-5348-A188-57E3FE2FE222}" name="Column1" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{06B06B16-BBC2-4F4E-A08E-BDFD62657B30}" name="model"/>
+    <tableColumn id="3" xr3:uid="{1DCE3343-5741-4246-B7F2-E351BFFA1384}" name="pipeline"/>
+    <tableColumn id="4" xr3:uid="{9B8CB705-14C5-DD4A-96C5-85CA2303A6FA}" name="compression"/>
+    <tableColumn id="5" xr3:uid="{78301DF2-CC9F-C741-B90A-388355849859}" name="attack"/>
+    <tableColumn id="6" xr3:uid="{749209FD-B225-AD4C-8E95-64807DB25E5C}" name="quality"/>
+    <tableColumn id="7" xr3:uid="{D57895CC-E688-9444-9E80-C5E73D6EE478}" name="epsilon"/>
+    <tableColumn id="8" xr3:uid="{39D62B7C-25AD-B847-9972-8C260C6B0EB7}" name="accuracy"/>
+    <tableColumn id="9" xr3:uid="{837AB921-9A8E-0145-8F68-DBE93E47EBAC}" name="correct"/>
+    <tableColumn id="10" xr3:uid="{2613A549-760C-4C43-818A-A9046078F6E0}" name="total"/>
+    <tableColumn id="11" xr3:uid="{08D1A4D9-AA93-464A-A4AC-F8AC3E43CDDF}" name="psnr_mean"/>
+    <tableColumn id="12" xr3:uid="{16D5207C-A05E-B242-8DB9-3E3DF91C742C}" name="mse_mean"/>
+    <tableColumn id="13" xr3:uid="{7CDE2A56-6DE1-F344-B566-5D12BB146849}" name="mae_mean"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -712,20 +823,23 @@
   <dimension ref="A1:M177"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="4.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.5" customWidth="1"/>
     <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" customWidth="1"/>
+    <col min="5" max="5" width="8.1640625" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
     <col min="7" max="7" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.83203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.83203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.1640625" customWidth="1"/>
+    <col min="9" max="9" width="9.1640625" customWidth="1"/>
+    <col min="10" max="10" width="7.1640625" customWidth="1"/>
     <col min="11" max="13" width="12.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>109</v>
+      </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -763,7 +877,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>0</v>
       </c>
@@ -792,7 +906,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -827,7 +941,7 @@
         <v>3.714720802903175E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -862,7 +976,7 @@
         <v>2.9169416984915729E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>3</v>
       </c>
@@ -897,7 +1011,7 @@
         <v>2.2731218534708018E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -932,7 +1046,7 @@
         <v>1.959524911642075E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>5</v>
       </c>
@@ -967,7 +1081,7 @@
         <v>5.6920524030923854E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>6</v>
       </c>
@@ -1002,7 +1116,7 @@
         <v>1.100760978460312E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>7</v>
       </c>
@@ -1037,7 +1151,7 @@
         <v>2.3005462104082108E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>8</v>
       </c>
@@ -1072,7 +1186,7 @@
         <v>6.3571486324071882E-3</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>9</v>
       </c>
@@ -1107,7 +1221,7 @@
         <v>1.2516078112646939E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>10</v>
       </c>
@@ -1142,7 +1256,7 @@
         <v>0.1622779815912247</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>11</v>
       </c>
@@ -1177,7 +1291,7 @@
         <v>0.10925147068500519</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>12</v>
       </c>
@@ -1212,7 +1326,7 @@
         <v>1.8634695428609849E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>13</v>
       </c>
@@ -1247,7 +1361,7 @@
         <v>3.0914242199063299E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>14</v>
       </c>
@@ -1282,7 +1396,7 @@
         <v>2.013240635693073E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>15</v>
       </c>
@@ -1317,7 +1431,7 @@
         <v>2.6477075758576388E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>16</v>
       </c>
@@ -1358,7 +1472,7 @@
         <v>4.6437945318222047E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>17</v>
       </c>
@@ -1399,7 +1513,7 @@
         <v>4.0672710758447653E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>18</v>
       </c>
@@ -1440,7 +1554,7 @@
         <v>3.6622209888696668E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>19</v>
       </c>
@@ -1481,7 +1595,7 @@
         <v>4.1558647966384893E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>20</v>
       </c>
@@ -1522,7 +1636,7 @@
         <v>3.4855703073740009E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>21</v>
       </c>
@@ -1563,7 +1677,7 @@
         <v>2.9925888854265208E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>22</v>
       </c>
@@ -1604,7 +1718,7 @@
         <v>4.4441168296337118E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>23</v>
       </c>
@@ -1645,7 +1759,7 @@
         <v>3.8479261922836301E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>24</v>
       </c>
@@ -1686,7 +1800,7 @@
         <v>3.4211361491680137E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>25</v>
       </c>
@@ -1727,7 +1841,7 @@
         <v>3.5264305007457732E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>26</v>
       </c>
@@ -1768,7 +1882,7 @@
         <v>3.100949060618877E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>27</v>
       </c>
@@ -1809,7 +1923,7 @@
         <v>3.0916062021255492E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
         <v>28</v>
       </c>
@@ -1850,7 +1964,7 @@
         <v>2.7985488152503971E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
         <v>29</v>
       </c>
@@ -1891,7 +2005,7 @@
         <v>2.0869215673208239E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
         <v>30</v>
       </c>
@@ -1932,7 +2046,7 @@
         <v>2.0181826800107959E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
         <v>31</v>
       </c>
@@ -1973,7 +2087,7 @@
         <v>3.2696889585256579E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
         <v>32</v>
       </c>
@@ -2014,7 +2128,7 @@
         <v>2.717305253148079E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
         <v>33</v>
       </c>
@@ -2055,7 +2169,7 @@
         <v>2.6568622708320621E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1">
         <v>34</v>
       </c>
@@ -2096,7 +2210,7 @@
         <v>3.8854352879524233E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
         <v>35</v>
       </c>
@@ -2137,7 +2251,7 @@
         <v>3.1242752081155779E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
         <v>36</v>
       </c>
@@ -2178,7 +2292,7 @@
         <v>3.0918344905972481E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" s="1">
         <v>37</v>
       </c>
@@ -2219,7 +2333,7 @@
         <v>3.1474095809459687E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>38</v>
       </c>
@@ -2260,7 +2374,7 @@
         <v>2.1306926387548449E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41" s="1">
         <v>39</v>
       </c>
@@ -2301,7 +2415,7 @@
         <v>2.0203948962688449E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
         <v>40</v>
       </c>
@@ -2342,7 +2456,7 @@
         <v>3.6002217531204223E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43" s="1">
         <v>41</v>
       </c>
@@ -2383,7 +2497,7 @@
         <v>2.7574413311481479E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44" s="1">
         <v>42</v>
       </c>
@@ -2424,7 +2538,7 @@
         <v>2.66580762386322E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" s="1">
         <v>43</v>
       </c>
@@ -2465,7 +2579,7 @@
         <v>0.1644177246570587</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" s="1">
         <v>44</v>
       </c>
@@ -2506,7 +2620,7 @@
         <v>0.1126609291434288</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47" s="1">
         <v>45</v>
       </c>
@@ -2547,7 +2661,7 @@
         <v>3.4225427126884457E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48" s="1">
         <v>46</v>
       </c>
@@ -2588,7 +2702,7 @@
         <v>0.16324073758125299</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A49" s="1">
         <v>47</v>
       </c>
@@ -2629,7 +2743,7 @@
         <v>0.11071992980241779</v>
       </c>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A50" s="1">
         <v>48</v>
       </c>
@@ -2670,7 +2784,7 @@
         <v>2.6996980729699131E-2</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51" s="1">
         <v>49</v>
       </c>
@@ -2711,7 +2825,7 @@
         <v>0.16368726823329929</v>
       </c>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A52" s="1">
         <v>50</v>
       </c>
@@ -2752,7 +2866,7 @@
         <v>0.11157314766645431</v>
       </c>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A53" s="1">
         <v>51</v>
       </c>
@@ -2793,7 +2907,7 @@
         <v>3.1791673034429549E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54" s="1">
         <v>52</v>
       </c>
@@ -2834,7 +2948,7 @@
         <v>3.8444789648056032E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A55" s="1">
         <v>53</v>
       </c>
@@ -2875,7 +2989,7 @@
         <v>3.1894125795364381E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A56" s="1">
         <v>54</v>
       </c>
@@ -2916,7 +3030,7 @@
         <v>2.933734335303307E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A57" s="1">
         <v>55</v>
       </c>
@@ -2957,7 +3071,7 @@
         <v>2.7087380433082581E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A58" s="1">
         <v>56</v>
       </c>
@@ -2998,7 +3112,7 @@
         <v>2.658754545450211E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A59" s="1">
         <v>57</v>
       </c>
@@ -3039,7 +3153,7 @@
         <v>3.0359493130445479E-2</v>
       </c>
     </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A60" s="1">
         <v>58</v>
       </c>
@@ -3080,7 +3194,7 @@
         <v>3.0740068498253819E-2</v>
       </c>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A61" s="1">
         <v>59</v>
       </c>
@@ -3121,7 +3235,7 @@
         <v>2.6756399676203729E-2</v>
       </c>
     </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A62" s="1">
         <v>60</v>
       </c>
@@ -3162,7 +3276,7 @@
         <v>3.022867523133755E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A63" s="1">
         <v>61</v>
       </c>
@@ -3203,7 +3317,7 @@
         <v>0.16230241889953609</v>
       </c>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A64" s="1">
         <v>62</v>
       </c>
@@ -3244,7 +3358,7 @@
         <v>0.1094397226333618</v>
       </c>
     </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A65" s="1">
         <v>63</v>
       </c>
@@ -3285,7 +3399,7 @@
         <v>2.7597814470529551E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A66" s="1">
         <v>64</v>
       </c>
@@ -3326,7 +3440,7 @@
         <v>3.7929028189182278E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A67" s="1">
         <v>65</v>
       </c>
@@ -3367,7 +3481,7 @@
         <v>3.0554869595170019E-2</v>
       </c>
     </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A68" s="1">
         <v>66</v>
       </c>
@@ -3408,7 +3522,7 @@
         <v>2.5496912685036659E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A69" s="1">
         <v>67</v>
       </c>
@@ -3449,7 +3563,7 @@
         <v>2.4256987279653551E-2</v>
       </c>
     </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A70" s="1">
         <v>68</v>
       </c>
@@ -3490,7 +3604,7 @@
         <v>1.8954976630210871E-2</v>
       </c>
     </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A71" s="1">
         <v>69</v>
       </c>
@@ -3531,7 +3645,7 @@
         <v>1.9967742916941641E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A72" s="1">
         <v>70</v>
       </c>
@@ -3572,7 +3686,7 @@
         <v>2.792199927568436E-2</v>
       </c>
     </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A73" s="1">
         <v>71</v>
       </c>
@@ -3613,7 +3727,7 @@
         <v>1.940122195482254E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A74" s="1">
         <v>72</v>
       </c>
@@ -3654,7 +3768,7 @@
         <v>1.9944944480061531E-2</v>
       </c>
     </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A75" s="1">
         <v>73</v>
       </c>
@@ -3695,7 +3809,7 @@
         <v>0.16231315221786499</v>
       </c>
     </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A76" s="1">
         <v>74</v>
       </c>
@@ -3736,7 +3850,7 @@
         <v>0.10939558382034301</v>
       </c>
     </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A77" s="1">
         <v>75</v>
       </c>
@@ -3779,98 +3893,98 @@
     </row>
     <row r="78" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A78" s="1">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="B78" t="s">
         <v>12</v>
       </c>
       <c r="C78" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="D78" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E78" t="s">
         <v>35</v>
       </c>
       <c r="F78">
-        <v>25</v>
+        <v>75</v>
       </c>
       <c r="G78">
         <v>3.1372549019607843E-2</v>
       </c>
       <c r="H78">
-        <v>0.55600000000000005</v>
+        <v>8.9999999999999998E-4</v>
       </c>
       <c r="I78">
-        <v>5560</v>
+        <v>9</v>
       </c>
       <c r="J78">
         <v>10000</v>
       </c>
       <c r="K78">
-        <v>26.068632946777349</v>
+        <v>31.055893096923828</v>
       </c>
       <c r="L78">
-        <v>2.6898837558925149E-3</v>
+        <v>8.09959221817553E-4</v>
       </c>
       <c r="M78">
-        <v>3.8194546496868133E-2</v>
+        <v>2.6396099999547E-2</v>
       </c>
     </row>
     <row r="79" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A79" s="1">
-        <v>77</v>
+        <v>172</v>
       </c>
       <c r="B79" t="s">
-        <v>12</v>
+        <v>108</v>
       </c>
       <c r="C79" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="D79" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="E79" t="s">
         <v>35</v>
       </c>
       <c r="F79">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="G79">
         <v>3.1372549019607843E-2</v>
       </c>
       <c r="H79">
-        <v>0.62729999999999997</v>
+        <v>1.2999999999999999E-3</v>
       </c>
       <c r="I79">
-        <v>6273</v>
+        <v>13</v>
       </c>
       <c r="J79">
         <v>10000</v>
       </c>
       <c r="K79">
-        <v>27.861967639160159</v>
+        <v>31.169381964111331</v>
       </c>
       <c r="L79">
-        <v>1.794852092862129E-3</v>
+        <v>7.9085253942757843E-4</v>
       </c>
       <c r="M79">
-        <v>3.1133765637874601E-2</v>
+        <v>2.5850366008281708E-2</v>
       </c>
     </row>
     <row r="80" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A80" s="1">
-        <v>78</v>
+        <v>169</v>
       </c>
       <c r="B80" t="s">
-        <v>12</v>
+        <v>108</v>
       </c>
       <c r="C80" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="D80" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E80" t="s">
         <v>35</v>
@@ -3882,63 +3996,63 @@
         <v>3.1372549019607843E-2</v>
       </c>
       <c r="H80">
-        <v>0.51590000000000003</v>
+        <v>1.5E-3</v>
       </c>
       <c r="I80">
-        <v>5159</v>
+        <v>15</v>
       </c>
       <c r="J80">
         <v>10000</v>
       </c>
       <c r="K80">
-        <v>29.107364428710941</v>
+        <v>31.14248819885254</v>
       </c>
       <c r="L80">
-        <v>1.330882572941482E-3</v>
+        <v>7.9524069307371974E-4</v>
       </c>
       <c r="M80">
-        <v>2.7290054723620411E-2</v>
+        <v>2.6022638109326361E-2</v>
       </c>
     </row>
     <row r="81" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A81" s="1">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="B81" t="s">
         <v>12</v>
       </c>
       <c r="C81" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="D81" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="E81" t="s">
         <v>35</v>
       </c>
       <c r="F81">
-        <v>25</v>
+        <v>75</v>
       </c>
       <c r="G81">
         <v>3.1372549019607843E-2</v>
       </c>
       <c r="H81">
-        <v>0.35449999999999998</v>
+        <v>1.6000000000000001E-3</v>
       </c>
       <c r="I81">
-        <v>3545</v>
+        <v>16</v>
       </c>
       <c r="J81">
         <v>10000</v>
       </c>
       <c r="K81">
-        <v>29.67218823547363</v>
+        <v>31.0579477142334</v>
       </c>
       <c r="L81">
-        <v>1.195147455111146E-3</v>
+        <v>8.0945149995386605E-4</v>
       </c>
       <c r="M81">
-        <v>2.6224665671586989E-2</v>
+        <v>2.6296580293774609E-2</v>
       </c>
     </row>
     <row r="82" spans="1:13" x14ac:dyDescent="0.2">
@@ -3984,13 +4098,13 @@
     </row>
     <row r="83" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A83" s="1">
-        <v>81</v>
+        <v>168</v>
       </c>
       <c r="B83" t="s">
-        <v>12</v>
+        <v>108</v>
       </c>
       <c r="C83" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D83" t="s">
         <v>19</v>
@@ -3999,39 +4113,39 @@
         <v>35</v>
       </c>
       <c r="F83">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="G83">
         <v>3.1372549019607843E-2</v>
       </c>
       <c r="H83">
-        <v>8.9999999999999998E-4</v>
+        <v>4.2099999999999999E-2</v>
       </c>
       <c r="I83">
-        <v>9</v>
+        <v>421</v>
       </c>
       <c r="J83">
         <v>10000</v>
       </c>
       <c r="K83">
-        <v>31.055893096923828</v>
+        <v>31.351605261230471</v>
       </c>
       <c r="L83">
-        <v>8.09959221817553E-4</v>
+        <v>7.5703064780682327E-4</v>
       </c>
       <c r="M83">
-        <v>2.6396099999547E-2</v>
+        <v>2.3681877994537349E-2</v>
       </c>
     </row>
     <row r="84" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A84" s="1">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B84" t="s">
         <v>12</v>
       </c>
       <c r="C84" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D84" t="s">
         <v>23</v>
@@ -4040,36 +4154,36 @@
         <v>35</v>
       </c>
       <c r="F84">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="G84">
         <v>3.1372549019607843E-2</v>
       </c>
       <c r="H84">
-        <v>0.32800000000000001</v>
+        <v>6.1699999999999998E-2</v>
       </c>
       <c r="I84">
-        <v>3280</v>
+        <v>617</v>
       </c>
       <c r="J84">
         <v>10000</v>
       </c>
       <c r="K84">
-        <v>27.988963006591799</v>
+        <v>31.120317987060549</v>
       </c>
       <c r="L84">
-        <v>1.7672944683581591E-3</v>
+        <v>7.9590586461126807E-4</v>
       </c>
       <c r="M84">
-        <v>2.9848174169659611E-2</v>
+        <v>2.4180852276086809E-2</v>
       </c>
     </row>
     <row r="85" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A85" s="1">
-        <v>83</v>
+        <v>171</v>
       </c>
       <c r="B85" t="s">
-        <v>12</v>
+        <v>108</v>
       </c>
       <c r="C85" t="s">
         <v>103</v>
@@ -4087,71 +4201,71 @@
         <v>3.1372549019607843E-2</v>
       </c>
       <c r="H85">
-        <v>6.1699999999999998E-2</v>
+        <v>7.4899999999999994E-2</v>
       </c>
       <c r="I85">
-        <v>617</v>
+        <v>749</v>
       </c>
       <c r="J85">
         <v>10000</v>
       </c>
       <c r="K85">
-        <v>31.120317987060549</v>
+        <v>31.178060540771479</v>
       </c>
       <c r="L85">
-        <v>7.9590586461126807E-4</v>
+        <v>7.8655432565137746E-4</v>
       </c>
       <c r="M85">
-        <v>2.4180852276086809E-2</v>
+        <v>2.3981442055106161E-2</v>
       </c>
     </row>
     <row r="86" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A86" s="1">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B86" t="s">
         <v>12</v>
       </c>
       <c r="C86" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D86" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E86" t="s">
         <v>35</v>
       </c>
       <c r="F86">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="G86">
         <v>3.1372549019607843E-2</v>
       </c>
       <c r="H86">
-        <v>1.6000000000000001E-3</v>
+        <v>0.1154</v>
       </c>
       <c r="I86">
-        <v>16</v>
+        <v>1154</v>
       </c>
       <c r="J86">
         <v>10000</v>
       </c>
       <c r="K86">
-        <v>31.0579477142334</v>
+        <v>14.302603430175781</v>
       </c>
       <c r="L86">
-        <v>8.0945149995386605E-4</v>
+        <v>4.4278855413198467E-2</v>
       </c>
       <c r="M86">
-        <v>2.6296580293774609E-2</v>
+        <v>0.16228508775234221</v>
       </c>
     </row>
     <row r="87" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A87" s="1">
-        <v>85</v>
+        <v>173</v>
       </c>
       <c r="B87" t="s">
-        <v>12</v>
+        <v>108</v>
       </c>
       <c r="C87" t="s">
         <v>105</v>
@@ -4169,30 +4283,30 @@
         <v>3.1372549019607843E-2</v>
       </c>
       <c r="H87">
-        <v>0.1154</v>
+        <v>0.1356</v>
       </c>
       <c r="I87">
-        <v>1154</v>
+        <v>1356</v>
       </c>
       <c r="J87">
         <v>10000</v>
       </c>
       <c r="K87">
-        <v>14.302603430175781</v>
+        <v>14.30222497253418</v>
       </c>
       <c r="L87">
-        <v>4.4278855413198467E-2</v>
+        <v>4.427917809486389E-2</v>
       </c>
       <c r="M87">
-        <v>0.16228508775234221</v>
+        <v>0.1622752018928528</v>
       </c>
     </row>
     <row r="88" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A88" s="1">
-        <v>86</v>
+        <v>174</v>
       </c>
       <c r="B88" t="s">
-        <v>12</v>
+        <v>108</v>
       </c>
       <c r="C88" t="s">
         <v>106</v>
@@ -4210,33 +4324,33 @@
         <v>3.1372549019607843E-2</v>
       </c>
       <c r="H88">
-        <v>0.16439999999999999</v>
+        <v>0.16289999999999999</v>
       </c>
       <c r="I88">
-        <v>1644</v>
+        <v>1629</v>
       </c>
       <c r="J88">
         <v>10000</v>
       </c>
       <c r="K88">
-        <v>17.286528256225591</v>
+        <v>17.286456481933591</v>
       </c>
       <c r="L88">
-        <v>2.2275338393449778E-2</v>
+        <v>2.2278301286697388E-2</v>
       </c>
       <c r="M88">
-        <v>0.10940677468776699</v>
+        <v>0.1094122195482254</v>
       </c>
     </row>
     <row r="89" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A89" s="1">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B89" t="s">
         <v>12</v>
       </c>
       <c r="C89" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D89" t="s">
         <v>27</v>
@@ -4245,31 +4359,31 @@
         <v>35</v>
       </c>
       <c r="F89">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="G89">
         <v>3.1372549019607843E-2</v>
       </c>
       <c r="H89">
-        <v>0.37980000000000003</v>
+        <v>0.16439999999999999</v>
       </c>
       <c r="I89">
-        <v>3798</v>
+        <v>1644</v>
       </c>
       <c r="J89">
         <v>10000</v>
       </c>
       <c r="K89">
-        <v>29.539895089721679</v>
+        <v>17.286528256225591</v>
       </c>
       <c r="L89">
-        <v>1.1813691230490801E-3</v>
+        <v>2.2275338393449778E-2</v>
       </c>
       <c r="M89">
-        <v>2.6430593240261081E-2</v>
-      </c>
-    </row>
-    <row r="90" spans="1:13" x14ac:dyDescent="0.2">
+        <v>0.10940677468776699</v>
+      </c>
+    </row>
+    <row r="90" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A90" s="1">
         <v>88</v>
       </c>
@@ -4298,7 +4412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A91" s="1">
         <v>89</v>
       </c>
@@ -4333,7 +4447,7 @@
         <v>3.714720802903175E-2</v>
       </c>
     </row>
-    <row r="92" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A92" s="1">
         <v>90</v>
       </c>
@@ -4368,7 +4482,7 @@
         <v>2.9169416984915729E-2</v>
       </c>
     </row>
-    <row r="93" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A93" s="1">
         <v>91</v>
       </c>
@@ -4403,7 +4517,7 @@
         <v>2.2731218534708018E-2</v>
       </c>
     </row>
-    <row r="94" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A94" s="1">
         <v>92</v>
       </c>
@@ -4438,7 +4552,7 @@
         <v>1.959524911642075E-2</v>
       </c>
     </row>
-    <row r="95" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A95" s="1">
         <v>93</v>
       </c>
@@ -4473,7 +4587,7 @@
         <v>5.6920524030923854E-3</v>
       </c>
     </row>
-    <row r="96" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A96" s="1">
         <v>94</v>
       </c>
@@ -4508,7 +4622,7 @@
         <v>1.100760978460312E-3</v>
       </c>
     </row>
-    <row r="97" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A97" s="1">
         <v>95</v>
       </c>
@@ -4543,7 +4657,7 @@
         <v>2.3005462104082108E-2</v>
       </c>
     </row>
-    <row r="98" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A98" s="1">
         <v>96</v>
       </c>
@@ -4578,7 +4692,7 @@
         <v>6.3571486324071882E-3</v>
       </c>
     </row>
-    <row r="99" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A99" s="1">
         <v>97</v>
       </c>
@@ -4613,7 +4727,7 @@
         <v>1.2516078112646939E-3</v>
       </c>
     </row>
-    <row r="100" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A100" s="1">
         <v>98</v>
       </c>
@@ -4648,7 +4762,7 @@
         <v>0.1622779815912247</v>
       </c>
     </row>
-    <row r="101" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A101" s="1">
         <v>99</v>
       </c>
@@ -4683,7 +4797,7 @@
         <v>0.10925147068500519</v>
       </c>
     </row>
-    <row r="102" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A102" s="1">
         <v>100</v>
       </c>
@@ -4718,7 +4832,7 @@
         <v>1.8634695428609849E-2</v>
       </c>
     </row>
-    <row r="103" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A103" s="1">
         <v>101</v>
       </c>
@@ -4753,7 +4867,7 @@
         <v>3.0915326565504071E-2</v>
       </c>
     </row>
-    <row r="104" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A104" s="1">
         <v>102</v>
       </c>
@@ -4788,7 +4902,7 @@
         <v>1.9593514624238011E-2</v>
       </c>
     </row>
-    <row r="105" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A105" s="1">
         <v>103</v>
       </c>
@@ -4823,7 +4937,7 @@
         <v>2.6015012633800509E-2</v>
       </c>
     </row>
-    <row r="106" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A106" s="1">
         <v>104</v>
       </c>
@@ -4864,7 +4978,7 @@
         <v>4.6434428775310517E-2</v>
       </c>
     </row>
-    <row r="107" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A107" s="1">
         <v>105</v>
       </c>
@@ -4905,7 +5019,7 @@
         <v>4.0669619470834729E-2</v>
       </c>
     </row>
-    <row r="108" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A108" s="1">
         <v>106</v>
       </c>
@@ -4946,7 +5060,7 @@
         <v>3.6668582010269173E-2</v>
       </c>
     </row>
-    <row r="109" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A109" s="1">
         <v>107</v>
       </c>
@@ -4987,7 +5101,7 @@
         <v>4.1359855079650877E-2</v>
       </c>
     </row>
-    <row r="110" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A110" s="1">
         <v>108</v>
       </c>
@@ -5028,7 +5142,7 @@
         <v>3.4585721921920783E-2</v>
       </c>
     </row>
-    <row r="111" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A111" s="1">
         <v>109</v>
       </c>
@@ -5069,7 +5183,7 @@
         <v>2.9566403681039809E-2</v>
       </c>
     </row>
-    <row r="112" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A112" s="1">
         <v>110</v>
       </c>
@@ -5110,7 +5224,7 @@
         <v>4.4257586616277697E-2</v>
       </c>
     </row>
-    <row r="113" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A113" s="1">
         <v>111</v>
       </c>
@@ -5151,7 +5265,7 @@
         <v>3.8177348613739011E-2</v>
       </c>
     </row>
-    <row r="114" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A114" s="1">
         <v>112</v>
       </c>
@@ -5192,7 +5306,7 @@
         <v>3.3919685828685757E-2</v>
       </c>
     </row>
-    <row r="115" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A115" s="1">
         <v>113</v>
       </c>
@@ -5233,7 +5347,7 @@
         <v>3.529983329772949E-2</v>
       </c>
     </row>
-    <row r="116" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A116" s="1">
         <v>114</v>
       </c>
@@ -5274,7 +5388,7 @@
         <v>3.103720471560955E-2</v>
       </c>
     </row>
-    <row r="117" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A117" s="1">
         <v>115</v>
       </c>
@@ -5315,7 +5429,7 @@
         <v>3.0920980742573739E-2</v>
       </c>
     </row>
-    <row r="118" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A118" s="1">
         <v>116</v>
       </c>
@@ -5356,7 +5470,7 @@
         <v>2.7619557735323909E-2</v>
       </c>
     </row>
-    <row r="119" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A119" s="1">
         <v>117</v>
       </c>
@@ -5397,7 +5511,7 @@
         <v>2.0355087161064149E-2</v>
       </c>
     </row>
-    <row r="120" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A120" s="1">
         <v>118</v>
       </c>
@@ -5438,7 +5552,7 @@
         <v>1.9640436738729481E-2</v>
       </c>
     </row>
-    <row r="121" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A121" s="1">
         <v>119</v>
       </c>
@@ -5479,7 +5593,7 @@
         <v>3.2273396056890488E-2</v>
       </c>
     </row>
-    <row r="122" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A122" s="1">
         <v>120</v>
       </c>
@@ -5520,7 +5634,7 @@
         <v>2.686941384673119E-2</v>
       </c>
     </row>
-    <row r="123" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A123" s="1">
         <v>121</v>
       </c>
@@ -5561,7 +5675,7 @@
         <v>2.6219588631391521E-2</v>
       </c>
     </row>
-    <row r="124" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A124" s="1">
         <v>122</v>
       </c>
@@ -5602,7 +5716,7 @@
         <v>3.888193833231926E-2</v>
       </c>
     </row>
-    <row r="125" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A125" s="1">
         <v>123</v>
       </c>
@@ -5643,7 +5757,7 @@
         <v>3.1271762835979461E-2</v>
       </c>
     </row>
-    <row r="126" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A126" s="1">
         <v>124</v>
       </c>
@@ -5684,7 +5798,7 @@
         <v>3.092154369652271E-2</v>
       </c>
     </row>
-    <row r="127" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A127" s="1">
         <v>125</v>
       </c>
@@ -5725,7 +5839,7 @@
         <v>3.1135721838474271E-2</v>
       </c>
     </row>
-    <row r="128" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A128" s="1">
         <v>126</v>
       </c>
@@ -5766,7 +5880,7 @@
         <v>2.079511488676071E-2</v>
       </c>
     </row>
-    <row r="129" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A129" s="1">
         <v>127</v>
       </c>
@@ -5807,7 +5921,7 @@
         <v>1.966359099447727E-2</v>
       </c>
     </row>
-    <row r="130" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A130" s="1">
         <v>128</v>
       </c>
@@ -5848,7 +5962,7 @@
         <v>3.549525844454765E-2</v>
       </c>
     </row>
-    <row r="131" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A131" s="1">
         <v>129</v>
       </c>
@@ -5889,7 +6003,7 @@
         <v>2.7178101712465291E-2</v>
       </c>
     </row>
-    <row r="132" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A132" s="1">
         <v>130</v>
       </c>
@@ -5930,7 +6044,7 @@
         <v>2.6182470220327381E-2</v>
       </c>
     </row>
-    <row r="133" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A133" s="1">
         <v>131</v>
       </c>
@@ -5971,7 +6085,7 @@
         <v>0.16437765452861791</v>
       </c>
     </row>
-    <row r="134" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A134" s="1">
         <v>132</v>
       </c>
@@ -6012,7 +6126,7 @@
         <v>0.11264622384309771</v>
       </c>
     </row>
-    <row r="135" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A135" s="1">
         <v>133</v>
       </c>
@@ -6053,7 +6167,7 @@
         <v>3.424507606625557E-2</v>
       </c>
     </row>
-    <row r="136" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A136" s="1">
         <v>134</v>
       </c>
@@ -6094,7 +6208,7 @@
         <v>0.16316689794063571</v>
       </c>
     </row>
-    <row r="137" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A137" s="1">
         <v>135</v>
       </c>
@@ -6135,7 +6249,7 @@
         <v>0.1106666240215302</v>
       </c>
     </row>
-    <row r="138" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A138" s="1">
         <v>136</v>
       </c>
@@ -6176,7 +6290,7 @@
         <v>2.6621283525228499E-2</v>
       </c>
     </row>
-    <row r="139" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A139" s="1">
         <v>137</v>
       </c>
@@ -6217,7 +6331,7 @@
         <v>0.16356636543273931</v>
       </c>
     </row>
-    <row r="140" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A140" s="1">
         <v>138</v>
       </c>
@@ -6258,7 +6372,7 @@
         <v>0.1113840122699738</v>
       </c>
     </row>
-    <row r="141" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A141" s="1">
         <v>139</v>
       </c>
@@ -6299,7 +6413,7 @@
         <v>3.1476817479729649E-2</v>
       </c>
     </row>
-    <row r="142" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A142" s="1">
         <v>140</v>
       </c>
@@ -6340,7 +6454,7 @@
         <v>3.8433512830734262E-2</v>
       </c>
     </row>
-    <row r="143" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A143" s="1">
         <v>141</v>
       </c>
@@ -6381,7 +6495,7 @@
         <v>3.1872253191471099E-2</v>
       </c>
     </row>
-    <row r="144" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A144" s="1">
         <v>142</v>
       </c>
@@ -6422,7 +6536,7 @@
         <v>2.9452684742212291E-2</v>
       </c>
     </row>
-    <row r="145" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A145" s="1">
         <v>143</v>
       </c>
@@ -6463,7 +6577,7 @@
         <v>2.7015410798788071E-2</v>
       </c>
     </row>
-    <row r="146" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A146" s="1">
         <v>144</v>
       </c>
@@ -6504,7 +6618,7 @@
         <v>2.6597175741195678E-2</v>
       </c>
     </row>
-    <row r="147" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A147" s="1">
         <v>145</v>
       </c>
@@ -6545,7 +6659,7 @@
         <v>3.03634593129158E-2</v>
       </c>
     </row>
-    <row r="148" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A148" s="1">
         <v>146</v>
       </c>
@@ -6586,7 +6700,7 @@
         <v>3.069180867373943E-2</v>
       </c>
     </row>
-    <row r="149" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A149" s="1">
         <v>147</v>
       </c>
@@ -6627,7 +6741,7 @@
         <v>2.6794984170794491E-2</v>
       </c>
     </row>
-    <row r="150" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A150" s="1">
         <v>148</v>
       </c>
@@ -6668,7 +6782,7 @@
         <v>3.0241151463985441E-2</v>
       </c>
     </row>
-    <row r="151" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A151" s="1">
         <v>149</v>
       </c>
@@ -6709,7 +6823,7 @@
         <v>0.16237861988544461</v>
       </c>
     </row>
-    <row r="152" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A152" s="1">
         <v>150</v>
       </c>
@@ -6750,7 +6864,7 @@
         <v>0.10936691430807111</v>
       </c>
     </row>
-    <row r="153" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A153" s="1">
         <v>151</v>
       </c>
@@ -6791,7 +6905,7 @@
         <v>2.7625030171871189E-2</v>
       </c>
     </row>
-    <row r="154" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A154" s="1">
         <v>152</v>
       </c>
@@ -6832,7 +6946,7 @@
         <v>3.7899359422922142E-2</v>
       </c>
     </row>
-    <row r="155" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A155" s="1">
         <v>153</v>
       </c>
@@ -6873,7 +6987,7 @@
         <v>3.050710678398609E-2</v>
       </c>
     </row>
-    <row r="156" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A156" s="1">
         <v>154</v>
       </c>
@@ -6914,7 +7028,7 @@
         <v>2.5378445443511009E-2</v>
       </c>
     </row>
-    <row r="157" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A157" s="1">
         <v>155</v>
       </c>
@@ -6955,7 +7069,7 @@
         <v>2.4015038102865219E-2</v>
       </c>
     </row>
-    <row r="158" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A158" s="1">
         <v>156</v>
       </c>
@@ -6996,7 +7110,7 @@
         <v>1.8519916605949399E-2</v>
       </c>
     </row>
-    <row r="159" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A159" s="1">
         <v>157</v>
       </c>
@@ -7037,7 +7151,7 @@
         <v>1.9422525417804721E-2</v>
       </c>
     </row>
-    <row r="160" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A160" s="1">
         <v>158</v>
       </c>
@@ -7078,7 +7192,7 @@
         <v>2.7705191159248351E-2</v>
       </c>
     </row>
-    <row r="161" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A161" s="1">
         <v>159</v>
       </c>
@@ -7119,7 +7233,7 @@
         <v>1.8985592848062519E-2</v>
       </c>
     </row>
-    <row r="162" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A162" s="1">
         <v>160</v>
       </c>
@@ -7160,7 +7274,7 @@
         <v>1.9414260572195051E-2</v>
       </c>
     </row>
-    <row r="163" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A163" s="1">
         <v>161</v>
       </c>
@@ -7201,7 +7315,7 @@
         <v>0.1623309042930603</v>
       </c>
     </row>
-    <row r="164" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A164" s="1">
         <v>162</v>
       </c>
@@ -7242,7 +7356,7 @@
         <v>0.10936690247058869</v>
       </c>
     </row>
-    <row r="165" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A165" s="1">
         <v>163</v>
       </c>
@@ -7285,16 +7399,16 @@
     </row>
     <row r="166" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A166" s="1">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="B166" t="s">
         <v>108</v>
       </c>
       <c r="C166" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D166" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="E166" t="s">
         <v>35</v>
@@ -7306,104 +7420,104 @@
         <v>3.1372549019607843E-2</v>
       </c>
       <c r="H166">
-        <v>0.58350000000000002</v>
+        <v>0.3115</v>
       </c>
       <c r="I166">
-        <v>5835</v>
+        <v>3115</v>
       </c>
       <c r="J166">
         <v>10000</v>
       </c>
       <c r="K166">
-        <v>26.076904019165038</v>
+        <v>28.02128120117187</v>
       </c>
       <c r="L166">
-        <v>2.6860524348914618E-3</v>
+        <v>1.7563372515141959E-3</v>
       </c>
       <c r="M166">
-        <v>3.8151044756174091E-2</v>
+        <v>2.9707281979918478E-2</v>
       </c>
     </row>
     <row r="167" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A167" s="1">
-        <v>165</v>
+        <v>82</v>
       </c>
       <c r="B167" t="s">
-        <v>108</v>
+        <v>12</v>
       </c>
       <c r="C167" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="D167" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="E167" t="s">
         <v>35</v>
       </c>
       <c r="F167">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="G167">
         <v>3.1372549019607843E-2</v>
       </c>
       <c r="H167">
-        <v>0.63849999999999996</v>
+        <v>0.32800000000000001</v>
       </c>
       <c r="I167">
-        <v>6385</v>
+        <v>3280</v>
       </c>
       <c r="J167">
         <v>10000</v>
       </c>
       <c r="K167">
-        <v>27.871696661376951</v>
+        <v>27.988963006591799</v>
       </c>
       <c r="L167">
-        <v>1.7920146774500611E-3</v>
+        <v>1.7672944683581591E-3</v>
       </c>
       <c r="M167">
-        <v>3.1082099175453189E-2</v>
+        <v>2.9848174169659611E-2</v>
       </c>
     </row>
     <row r="168" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A168" s="1">
-        <v>166</v>
+        <v>79</v>
       </c>
       <c r="B168" t="s">
-        <v>108</v>
+        <v>12</v>
       </c>
       <c r="C168" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D168" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E168" t="s">
         <v>35</v>
       </c>
       <c r="F168">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="G168">
         <v>3.1372549019607843E-2</v>
       </c>
       <c r="H168">
-        <v>0.49340000000000001</v>
+        <v>0.35449999999999998</v>
       </c>
       <c r="I168">
-        <v>4934</v>
+        <v>3545</v>
       </c>
       <c r="J168">
         <v>10000</v>
       </c>
       <c r="K168">
-        <v>29.079194515991212</v>
+        <v>29.67218823547363</v>
       </c>
       <c r="L168">
-        <v>1.3380954397842291E-3</v>
+        <v>1.195147455111146E-3</v>
       </c>
       <c r="M168">
-        <v>2.737296213507652E-2</v>
+        <v>2.6224665671586989E-2</v>
       </c>
     </row>
     <row r="169" spans="1:13" x14ac:dyDescent="0.2">
@@ -7449,57 +7563,57 @@
     </row>
     <row r="170" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A170" s="1">
-        <v>168</v>
+        <v>87</v>
       </c>
       <c r="B170" t="s">
-        <v>108</v>
+        <v>12</v>
       </c>
       <c r="C170" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="D170" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="E170" t="s">
         <v>35</v>
       </c>
       <c r="F170">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="G170">
         <v>3.1372549019607843E-2</v>
       </c>
       <c r="H170">
-        <v>4.2099999999999999E-2</v>
+        <v>0.37980000000000003</v>
       </c>
       <c r="I170">
-        <v>421</v>
+        <v>3798</v>
       </c>
       <c r="J170">
         <v>10000</v>
       </c>
       <c r="K170">
-        <v>31.351605261230471</v>
+        <v>29.539895089721679</v>
       </c>
       <c r="L170">
-        <v>7.5703064780682327E-4</v>
+        <v>1.1813691230490801E-3</v>
       </c>
       <c r="M170">
-        <v>2.3681877994537349E-2</v>
+        <v>2.6430593240261081E-2</v>
       </c>
     </row>
     <row r="171" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A171" s="1">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="B171" t="s">
         <v>108</v>
       </c>
       <c r="C171" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="D171" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="E171" t="s">
         <v>35</v>
@@ -7511,159 +7625,159 @@
         <v>3.1372549019607843E-2</v>
       </c>
       <c r="H171">
-        <v>1.5E-3</v>
+        <v>0.41959999999999997</v>
       </c>
       <c r="I171">
-        <v>15</v>
+        <v>4196</v>
       </c>
       <c r="J171">
         <v>10000</v>
       </c>
       <c r="K171">
-        <v>31.14248819885254</v>
+        <v>29.61537376403809</v>
       </c>
       <c r="L171">
-        <v>7.9524069307371974E-4</v>
+        <v>1.166154735162854E-3</v>
       </c>
       <c r="M171">
-        <v>2.6022638109326361E-2</v>
+        <v>2.6194074225425721E-2</v>
       </c>
     </row>
     <row r="172" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A172" s="1">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B172" t="s">
         <v>108</v>
       </c>
       <c r="C172" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="D172" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="E172" t="s">
         <v>35</v>
       </c>
       <c r="F172">
-        <v>25</v>
+        <v>75</v>
       </c>
       <c r="G172">
         <v>3.1372549019607843E-2</v>
       </c>
       <c r="H172">
-        <v>0.3115</v>
+        <v>0.49340000000000001</v>
       </c>
       <c r="I172">
-        <v>3115</v>
+        <v>4934</v>
       </c>
       <c r="J172">
         <v>10000</v>
       </c>
       <c r="K172">
-        <v>28.02128120117187</v>
+        <v>29.079194515991212</v>
       </c>
       <c r="L172">
-        <v>1.7563372515141959E-3</v>
+        <v>1.3380954397842291E-3</v>
       </c>
       <c r="M172">
-        <v>2.9707281979918478E-2</v>
+        <v>2.737296213507652E-2</v>
       </c>
     </row>
     <row r="173" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A173" s="1">
-        <v>171</v>
+        <v>78</v>
       </c>
       <c r="B173" t="s">
-        <v>108</v>
+        <v>12</v>
       </c>
       <c r="C173" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="D173" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="E173" t="s">
         <v>35</v>
       </c>
       <c r="F173">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="G173">
         <v>3.1372549019607843E-2</v>
       </c>
       <c r="H173">
-        <v>7.4899999999999994E-2</v>
+        <v>0.51590000000000003</v>
       </c>
       <c r="I173">
-        <v>749</v>
+        <v>5159</v>
       </c>
       <c r="J173">
         <v>10000</v>
       </c>
       <c r="K173">
-        <v>31.178060540771479</v>
+        <v>29.107364428710941</v>
       </c>
       <c r="L173">
-        <v>7.8655432565137746E-4</v>
+        <v>1.330882572941482E-3</v>
       </c>
       <c r="M173">
-        <v>2.3981442055106161E-2</v>
+        <v>2.7290054723620411E-2</v>
       </c>
     </row>
     <row r="174" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A174" s="1">
-        <v>172</v>
+        <v>76</v>
       </c>
       <c r="B174" t="s">
-        <v>108</v>
+        <v>12</v>
       </c>
       <c r="C174" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="D174" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="E174" t="s">
         <v>35</v>
       </c>
       <c r="F174">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="G174">
         <v>3.1372549019607843E-2</v>
       </c>
       <c r="H174">
-        <v>1.2999999999999999E-3</v>
+        <v>0.55600000000000005</v>
       </c>
       <c r="I174">
-        <v>13</v>
+        <v>5560</v>
       </c>
       <c r="J174">
         <v>10000</v>
       </c>
       <c r="K174">
-        <v>31.169381964111331</v>
+        <v>26.068632946777349</v>
       </c>
       <c r="L174">
-        <v>7.9085253942757843E-4</v>
+        <v>2.6898837558925149E-3</v>
       </c>
       <c r="M174">
-        <v>2.5850366008281708E-2</v>
+        <v>3.8194546496868133E-2</v>
       </c>
     </row>
     <row r="175" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A175" s="1">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="B175" t="s">
         <v>108</v>
       </c>
       <c r="C175" t="s">
-        <v>105</v>
+        <v>96</v>
       </c>
       <c r="D175" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="E175" t="s">
         <v>35</v>
@@ -7675,36 +7789,36 @@
         <v>3.1372549019607843E-2</v>
       </c>
       <c r="H175">
-        <v>0.1356</v>
+        <v>0.58350000000000002</v>
       </c>
       <c r="I175">
-        <v>1356</v>
+        <v>5835</v>
       </c>
       <c r="J175">
         <v>10000</v>
       </c>
       <c r="K175">
-        <v>14.30222497253418</v>
+        <v>26.076904019165038</v>
       </c>
       <c r="L175">
-        <v>4.427917809486389E-2</v>
+        <v>2.6860524348914618E-3</v>
       </c>
       <c r="M175">
-        <v>0.1622752018928528</v>
+        <v>3.8151044756174091E-2</v>
       </c>
     </row>
     <row r="176" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A176" s="1">
-        <v>174</v>
+        <v>77</v>
       </c>
       <c r="B176" t="s">
-        <v>108</v>
+        <v>12</v>
       </c>
       <c r="C176" t="s">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="D176" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="E176" t="s">
         <v>35</v>
@@ -7716,66 +7830,69 @@
         <v>3.1372549019607843E-2</v>
       </c>
       <c r="H176">
-        <v>0.16289999999999999</v>
+        <v>0.62729999999999997</v>
       </c>
       <c r="I176">
-        <v>1629</v>
+        <v>6273</v>
       </c>
       <c r="J176">
         <v>10000</v>
       </c>
       <c r="K176">
-        <v>17.286456481933591</v>
+        <v>27.861967639160159</v>
       </c>
       <c r="L176">
-        <v>2.2278301286697388E-2</v>
+        <v>1.794852092862129E-3</v>
       </c>
       <c r="M176">
-        <v>0.1094122195482254</v>
+        <v>3.1133765637874601E-2</v>
       </c>
     </row>
     <row r="177" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A177" s="1">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="B177" t="s">
         <v>108</v>
       </c>
       <c r="C177" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="D177" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="E177" t="s">
         <v>35</v>
       </c>
       <c r="F177">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="G177">
         <v>3.1372549019607843E-2</v>
       </c>
       <c r="H177">
-        <v>0.41959999999999997</v>
+        <v>0.63849999999999996</v>
       </c>
       <c r="I177">
-        <v>4196</v>
+        <v>6385</v>
       </c>
       <c r="J177">
         <v>10000</v>
       </c>
       <c r="K177">
-        <v>29.61537376403809</v>
+        <v>27.871696661376951</v>
       </c>
       <c r="L177">
-        <v>1.166154735162854E-3</v>
+        <v>1.7920146774500611E-3</v>
       </c>
       <c r="M177">
-        <v>2.6194074225425721E-2</v>
+        <v>3.1082099175453189E-2</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>